<commit_message>
chore: update CAN data mappings in Blue01_M_CAN_4836.xlsx
</commit_message>
<xml_diff>
--- a/Blue01_M_CAN_4836.xlsx
+++ b/Blue01_M_CAN_4836.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC4C7301-3C79-4C7D-BA75-F1D7BA51935E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9F40C8-8C55-4A23-B9DE-684B91A1C857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protocol" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,148 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="168">
+  <si>
+    <t>id_or_address</t>
+  </si>
+  <si>
+    <t>signal_name</t>
+  </si>
+  <si>
+    <t>bit_index</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>0x2F9</t>
+  </si>
+  <si>
+    <t>Contactor_Status</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Precharge Relay</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Main Contactor</t>
+  </si>
+  <si>
+    <t>0x1F0</t>
+  </si>
+  <si>
+    <t>System_Faults</t>
+  </si>
+  <si>
+    <t>Cell Over Voltage (COV)</t>
+  </si>
+  <si>
+    <t>Cell Under Voltage (CUV)</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Pack Over Voltage (POV)</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Pack Under Voltage (PUV)</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Cell Over Temperature (COT)</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Cell Under Temperature (CUT)</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Over Current Charge (OCC)</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Over Current Discharge (OCD)</t>
+  </si>
+  <si>
+    <t>Balancing_Status</t>
+  </si>
+  <si>
+    <t>Cell 1 Status</t>
+  </si>
+  <si>
+    <t>Cell 2 Status</t>
+  </si>
+  <si>
+    <t>Cell 3 Status</t>
+  </si>
+  <si>
+    <t>Cell 4 Status</t>
+  </si>
+  <si>
+    <t>Cell 5 Status</t>
+  </si>
+  <si>
+    <t>Cell 6 Status</t>
+  </si>
+  <si>
+    <t>Cell 7 Status</t>
+  </si>
+  <si>
+    <t>Cell 8 Status</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Cell 9 Status</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Cell 10 Status</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Cell 11 Status</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Cell 12 Status</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Cell 13 Status</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Cell 14 Status</t>
+  </si>
   <si>
     <t>profile_name</t>
   </si>
@@ -84,33 +225,21 @@
     <t>AA</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>little</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>payload_only</t>
   </si>
   <si>
     <t>none</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>55</t>
   </si>
   <si>
     <t>hex</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>True</t>
   </si>
   <si>
@@ -165,24 +294,30 @@
     <t>0x2F5</t>
   </si>
   <si>
+    <t>BMS_AFE_And_Pack_Temperatures_1_3</t>
+  </si>
+  <si>
     <t>0x2F6</t>
   </si>
   <si>
+    <t>BMS_Pack_Temperatures_4_7</t>
+  </si>
+  <si>
     <t>0x2F7</t>
   </si>
   <si>
+    <t>BMS_BR_Temperatures_1_3</t>
+  </si>
+  <si>
     <t>0x2F8</t>
   </si>
   <si>
-    <t>0x2F9</t>
+    <t>BMS_PCR_BDPS_1_2_And_A_Temperature</t>
   </si>
   <si>
     <t>BMS_Contactor_Management</t>
   </si>
   <si>
-    <t>0x1F0</t>
-  </si>
-  <si>
     <t>BMS_Faults_And_Status</t>
   </si>
   <si>
@@ -198,12 +333,6 @@
     <t>BMS_State_Capacity</t>
   </si>
   <si>
-    <t>id_or_address</t>
-  </si>
-  <si>
-    <t>signal_name</t>
-  </si>
-  <si>
     <t>data_type</t>
   </si>
   <si>
@@ -252,9 +381,6 @@
     <t>R</t>
   </si>
   <si>
-    <t>4294967295</t>
-  </si>
-  <si>
     <t>Pack_Current</t>
   </si>
   <si>
@@ -264,12 +390,6 @@
     <t>A</t>
   </si>
   <si>
-    <t>-2147483648</t>
-  </si>
-  <si>
-    <t>2147483647</t>
-  </si>
-  <si>
     <t>Cell_Voltage</t>
   </si>
   <si>
@@ -279,12 +399,6 @@
     <t>Cell Voltages</t>
   </si>
   <si>
-    <t>2000</t>
-  </si>
-  <si>
-    <t>4500</t>
-  </si>
-  <si>
     <t>AFE_Temperature</t>
   </si>
   <si>
@@ -297,234 +411,96 @@
     <t>AFE Temperatures</t>
   </si>
   <si>
-    <t>-40</t>
+    <t>Pack_Temperature</t>
+  </si>
+  <si>
+    <t>Pack Temperatures</t>
+  </si>
+  <si>
+    <t>Balancing_Resistor_Temperature</t>
+  </si>
+  <si>
+    <t>Precharge_Resistor_Temperature</t>
+  </si>
+  <si>
+    <t>Bidirectional_Power_Switch_Temperature</t>
+  </si>
+  <si>
+    <t>Ambient_Temperature</t>
+  </si>
+  <si>
+    <t>Load_Voltage</t>
+  </si>
+  <si>
+    <t>uint8</t>
+  </si>
+  <si>
+    <t>BitFields</t>
+  </si>
+  <si>
+    <t>Faults and Alarms</t>
+  </si>
+  <si>
+    <t>Balancing Status</t>
+  </si>
+  <si>
+    <t>BMS_Operation_State</t>
+  </si>
+  <si>
+    <t>Enums</t>
+  </si>
+  <si>
+    <t>Operation State</t>
+  </si>
+  <si>
+    <t>OCV_SOC</t>
+  </si>
+  <si>
+    <t>single</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>SOC</t>
+  </si>
+  <si>
+    <t>CC_SOC</t>
+  </si>
+  <si>
+    <t>State_Capacity</t>
+  </si>
+  <si>
+    <t>Ah</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>baud_rate</t>
+  </si>
+  <si>
+    <t>data_bits</t>
+  </si>
+  <si>
+    <t>stop_bits</t>
+  </si>
+  <si>
+    <t>parity</t>
+  </si>
+  <si>
+    <t>timeout_ms</t>
+  </si>
+  <si>
+    <t>2000000</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
   <si>
     <t>100</t>
   </si>
   <si>
-    <t>Pack_Temperature</t>
-  </si>
-  <si>
-    <t>Pack Temperatures</t>
-  </si>
-  <si>
-    <t>-50</t>
-  </si>
-  <si>
-    <t>150</t>
-  </si>
-  <si>
-    <t>Balancing_Resistor_Temperature</t>
-  </si>
-  <si>
-    <t>Precharge_Resistor_Temperature</t>
-  </si>
-  <si>
-    <t>Bidirectional_Power_Switch_Temperature</t>
-  </si>
-  <si>
-    <t>Contactor_Status</t>
-  </si>
-  <si>
-    <t>uint8</t>
-  </si>
-  <si>
-    <t>BitFields</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>System_Faults</t>
-  </si>
-  <si>
-    <t>Faults and Alarms</t>
-  </si>
-  <si>
-    <t>Balancing_Status</t>
-  </si>
-  <si>
-    <t>Balancing Status</t>
-  </si>
-  <si>
-    <t>BMS_Operation_State</t>
-  </si>
-  <si>
-    <t>Enums</t>
-  </si>
-  <si>
-    <t>Operation State</t>
-  </si>
-  <si>
-    <t>OCV_SOC</t>
-  </si>
-  <si>
-    <t>single</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>SOC</t>
-  </si>
-  <si>
-    <t>CC_SOC</t>
-  </si>
-  <si>
-    <t>State_Capacity</t>
-  </si>
-  <si>
-    <t>Ah</t>
-  </si>
-  <si>
-    <t>Capacity</t>
-  </si>
-  <si>
-    <t>``````</t>
-  </si>
-  <si>
-    <t>baud_rate</t>
-  </si>
-  <si>
-    <t>data_bits</t>
-  </si>
-  <si>
-    <t>stop_bits</t>
-  </si>
-  <si>
-    <t>parity</t>
-  </si>
-  <si>
-    <t>timeout_ms</t>
-  </si>
-  <si>
-    <t>2000000</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>bit_index</t>
-  </si>
-  <si>
-    <t>label</t>
-  </si>
-  <si>
-    <t>Precharge Relay</t>
-  </si>
-  <si>
-    <t>Main Contactor</t>
-  </si>
-  <si>
-    <t>Cell Over Voltage (COV)</t>
-  </si>
-  <si>
-    <t>Cell Under Voltage (CUV)</t>
-  </si>
-  <si>
-    <t>Pack Over Voltage (POV)</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Pack Under Voltage (PUV)</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Cell Over Temperature (COT)</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Cell Under Temperature (CUT)</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>Over Current Charge (OCC)</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>Over Current Discharge (OCD)</t>
-  </si>
-  <si>
-    <t>Cell 1 Status</t>
-  </si>
-  <si>
-    <t>Cell 2 Status</t>
-  </si>
-  <si>
-    <t>Cell 3 Status</t>
-  </si>
-  <si>
-    <t>Cell 4 Status</t>
-  </si>
-  <si>
-    <t>Cell 5 Status</t>
-  </si>
-  <si>
-    <t>Cell 6 Status</t>
-  </si>
-  <si>
-    <t>Cell 7 Status</t>
-  </si>
-  <si>
-    <t>Cell 8 Status</t>
-  </si>
-  <si>
-    <t>Cell 9 Status</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>Cell 10 Status</t>
-  </si>
-  <si>
-    <t>Cell 11 Status</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>Cell 12 Status</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>Cell 13 Status</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>Cell 14 Status</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Cell 15 Status</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Cell 16 Status</t>
-  </si>
-  <si>
     <t>value</t>
   </si>
   <si>
@@ -556,21 +532,6 @@
   </si>
   <si>
     <t>max|avg</t>
-  </si>
-  <si>
-    <t>BMS_AFE_And_Pack_Temperatures_1_3</t>
-  </si>
-  <si>
-    <t>BMS_Pack_Temperatures_4_7</t>
-  </si>
-  <si>
-    <t>BMS_PCR_And_BR_Temperatures_1_3</t>
-  </si>
-  <si>
-    <t>BMS_BDPST_1_2_And_A_Temperature</t>
-  </si>
-  <si>
-    <t>Ambient Temprature</t>
   </si>
 </sst>
 </file>
@@ -942,96 +903,96 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="K2" t="s">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="L2" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="M2" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="N2" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="O2" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1051,36 +1012,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="C2">
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -1088,16 +1049,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
       <c r="C3">
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -1105,16 +1066,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="C4">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -1122,16 +1083,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="C5">
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -1139,16 +1100,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>86</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -1156,16 +1117,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="B7" t="s">
-        <v>176</v>
+        <v>88</v>
       </c>
       <c r="C7">
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -1173,16 +1134,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>177</v>
+        <v>90</v>
       </c>
       <c r="C8">
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -1190,16 +1151,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>178</v>
+        <v>92</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -1207,16 +1168,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>179</v>
+        <v>94</v>
       </c>
       <c r="C10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -1224,16 +1185,16 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>95</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -1241,16 +1202,16 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="C12">
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -1258,16 +1219,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="C13">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -1275,16 +1236,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="C14">
         <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -1297,7 +1258,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
@@ -1318,66 +1279,66 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="O1" s="1" t="s">
-        <v>68</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F2">
         <v>1E-3</v>
@@ -1386,19 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="I2" t="s">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="J2" t="s">
-        <v>73</v>
-      </c>
-      <c r="K2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" t="s">
-        <v>74</v>
+        <v>116</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -1406,19 +1361,19 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F3">
         <v>1E-3</v>
@@ -1427,19 +1382,13 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>77</v>
+        <v>119</v>
       </c>
       <c r="I3" t="s">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
-      </c>
-      <c r="K3" t="s">
-        <v>78</v>
-      </c>
-      <c r="L3" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -1447,19 +1396,19 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D4">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F4">
         <v>1E-3</v>
@@ -1468,19 +1417,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="J4" t="s">
-        <v>73</v>
-      </c>
-      <c r="K4" t="s">
-        <v>83</v>
-      </c>
-      <c r="L4" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1491,19 +1434,19 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D5">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F5">
         <v>1E-3</v>
@@ -1512,19 +1455,13 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="I5" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
-      </c>
-      <c r="K5" t="s">
-        <v>83</v>
-      </c>
-      <c r="L5" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -1535,19 +1472,19 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D6">
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F6">
         <v>1E-3</v>
@@ -1556,19 +1493,13 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="I6" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="J6" t="s">
-        <v>73</v>
-      </c>
-      <c r="K6" t="s">
-        <v>83</v>
-      </c>
-      <c r="L6" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -1579,40 +1510,34 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F7">
         <v>1E-3</v>
       </c>
-      <c r="G7" t="s">
-        <v>23</v>
+      <c r="G7">
+        <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="I7" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="J7" t="s">
-        <v>73</v>
-      </c>
-      <c r="K7" t="s">
-        <v>83</v>
-      </c>
-      <c r="L7" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -1623,40 +1548,34 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>123</v>
       </c>
       <c r="C8" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F8">
         <v>0.1</v>
       </c>
-      <c r="G8" t="s">
-        <v>23</v>
+      <c r="G8">
+        <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I8" t="s">
-        <v>88</v>
+        <v>126</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
-      </c>
-      <c r="K8" t="s">
-        <v>89</v>
-      </c>
-      <c r="L8" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
@@ -1664,163 +1583,148 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="D9">
         <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F9">
         <v>0.1</v>
       </c>
-      <c r="G9" t="s">
-        <v>23</v>
+      <c r="G9">
+        <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I9" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K9" t="s">
-        <v>89</v>
-      </c>
-      <c r="L9" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D10">
         <v>4</v>
       </c>
       <c r="E10" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F10">
         <v>0.1</v>
       </c>
-      <c r="G10" t="s">
-        <v>23</v>
+      <c r="G10">
+        <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I10" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
-      </c>
-      <c r="K10" t="s">
-        <v>93</v>
-      </c>
-      <c r="L10" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
+      </c>
+      <c r="O10">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D11">
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F11">
         <v>0.1</v>
       </c>
-      <c r="G11" t="s">
-        <v>23</v>
+      <c r="G11">
+        <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I11" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="J11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K11" t="s">
-        <v>93</v>
-      </c>
-      <c r="L11" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="N11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F12">
         <v>0.1</v>
       </c>
-      <c r="G12" t="s">
-        <v>23</v>
+      <c r="G12">
+        <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I12" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="J12" t="s">
-        <v>73</v>
-      </c>
-      <c r="K12">
-        <v>-50</v>
-      </c>
-      <c r="L12" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="N12" t="b">
         <v>1</v>
@@ -1828,81 +1732,72 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>131</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="D13">
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F13">
         <v>0.1</v>
       </c>
-      <c r="G13" t="s">
-        <v>23</v>
+      <c r="G13">
+        <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I13" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
-      </c>
-      <c r="K13" t="s">
-        <v>89</v>
-      </c>
-      <c r="L13" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
-        <v>180</v>
+        <v>132</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F14">
         <v>0.1</v>
       </c>
-      <c r="G14" t="s">
-        <v>23</v>
+      <c r="G14">
+        <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="I14" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="J14" t="s">
-        <v>73</v>
-      </c>
-      <c r="K14" t="s">
-        <v>89</v>
-      </c>
-      <c r="L14" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
@@ -1910,40 +1805,34 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15" t="s">
-        <v>23</v>
+        <v>1E-3</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="I15" t="s">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="J15" t="s">
-        <v>73</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="N15" t="b">
         <v>1</v>
@@ -1951,37 +1840,34 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>102</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>134</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
-      <c r="G16" t="s">
-        <v>23</v>
+      <c r="G16">
+        <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>100</v>
+        <v>135</v>
       </c>
       <c r="I16" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="J16" t="s">
-        <v>73</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
@@ -1989,37 +1875,34 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
-      <c r="G17" t="s">
-        <v>23</v>
+      <c r="G17">
+        <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>100</v>
+        <v>135</v>
       </c>
       <c r="I17" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="J17" t="s">
-        <v>73</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
@@ -2027,19 +1910,19 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>106</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -2048,16 +1931,13 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="I18" t="s">
-        <v>108</v>
+        <v>137</v>
       </c>
       <c r="J18" t="s">
-        <v>73</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
@@ -2065,19 +1945,19 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -2086,16 +1966,13 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="I19" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="J19" t="s">
-        <v>73</v>
-      </c>
-      <c r="K19">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="N19" t="b">
         <v>1</v>
@@ -2103,19 +1980,19 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="B20" t="s">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>142</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -2124,16 +2001,13 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
       <c r="I20" t="s">
-        <v>112</v>
+        <v>144</v>
       </c>
       <c r="J20" t="s">
-        <v>73</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
@@ -2141,19 +2015,19 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>97</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>145</v>
       </c>
       <c r="C21" t="s">
-        <v>110</v>
+        <v>142</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -2162,24 +2036,51 @@
         <v>0</v>
       </c>
       <c r="H21" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="I21" t="s">
+        <v>144</v>
+      </c>
+      <c r="J21" t="s">
         <v>116</v>
       </c>
-      <c r="J21" t="s">
-        <v>73</v>
-      </c>
-      <c r="K21">
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C22" t="s">
+        <v>142</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
         <v>0</v>
       </c>
-      <c r="N21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="L24" t="s">
-        <v>117</v>
+      <c r="H22" t="s">
+        <v>147</v>
+      </c>
+      <c r="I22" t="s">
+        <v>148</v>
+      </c>
+      <c r="J22" t="s">
+        <v>116</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2194,36 +2095,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="E2" t="s">
-        <v>90</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -2233,7 +2134,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
@@ -2244,380 +2145,352 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>128</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>129</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>131</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>132</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>134</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>135</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>136</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>138</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>139</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>140</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>141</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>143</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>144</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>145</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>133</v>
+        <v>16</v>
       </c>
       <c r="D15" t="s">
-        <v>146</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>135</v>
+        <v>18</v>
       </c>
       <c r="D16" t="s">
-        <v>147</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>148</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>139</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>149</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C19" t="s">
-        <v>141</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
-        <v>150</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>124</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>151</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>152</v>
+        <v>37</v>
       </c>
       <c r="D21" t="s">
-        <v>153</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D22" t="s">
-        <v>154</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>155</v>
+        <v>41</v>
       </c>
       <c r="D23" t="s">
-        <v>156</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C24" t="s">
-        <v>157</v>
+        <v>43</v>
       </c>
       <c r="D24" t="s">
-        <v>158</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="C25" t="s">
-        <v>159</v>
+        <v>45</v>
       </c>
       <c r="D25" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" t="s">
-        <v>161</v>
-      </c>
-      <c r="D26" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>50</v>
-      </c>
-      <c r="B27" t="s">
-        <v>104</v>
-      </c>
-      <c r="C27" t="s">
-        <v>163</v>
-      </c>
-      <c r="D27" t="s">
-        <v>164</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -2638,58 +2511,58 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2711,19 +2584,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2748,31 +2621,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>67</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2791,34 +2664,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>126</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update Blue01_M_CAN_4836 dataset file
</commit_message>
<xml_diff>
--- a/Blue01_M_CAN_4836.xlsx
+++ b/Blue01_M_CAN_4836.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9F40C8-8C55-4A23-B9DE-684B91A1C857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D1A669-A2D7-4B35-82DD-11296675E5F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protocol" sheetId="1" r:id="rId1"/>
@@ -306,15 +306,9 @@
     <t>0x2F7</t>
   </si>
   <si>
-    <t>BMS_BR_Temperatures_1_3</t>
-  </si>
-  <si>
     <t>0x2F8</t>
   </si>
   <si>
-    <t>BMS_PCR_BDPS_1_2_And_A_Temperature</t>
-  </si>
-  <si>
     <t>BMS_Contactor_Management</t>
   </si>
   <si>
@@ -532,6 +526,12 @@
   </si>
   <si>
     <t>max|avg</t>
+  </si>
+  <si>
+    <t>BMS_BDPS_1_2_And_A_Temperature</t>
+  </si>
+  <si>
+    <t>BMS_BR_1_3_And_PCR_Temperatures</t>
   </si>
 </sst>
 </file>
@@ -1005,7 +1005,7 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40.26953125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1154,10 +1154,10 @@
         <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>167</v>
       </c>
       <c r="C9">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" t="s">
         <v>78</v>
@@ -1168,13 +1168,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D10" t="s">
         <v>78</v>
@@ -1188,7 +1188,7 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C11">
         <v>5</v>
@@ -1205,7 +1205,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C12">
         <v>3</v>
@@ -1219,10 +1219,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C13">
         <v>8</v>
@@ -1236,10 +1236,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C14">
         <v>4</v>
@@ -1285,34 +1285,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>75</v>
@@ -1321,7 +1321,7 @@
         <v>61</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
@@ -1329,10 +1329,10 @@
         <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I2" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" t="s">
         <v>114</v>
-      </c>
-      <c r="I2" t="s">
-        <v>115</v>
-      </c>
-      <c r="J2" t="s">
-        <v>116</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -1364,10 +1364,10 @@
         <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1382,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -1399,10 +1399,10 @@
         <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -1417,13 +1417,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I4" t="s">
+        <v>120</v>
+      </c>
+      <c r="J4" t="s">
         <v>114</v>
-      </c>
-      <c r="I4" t="s">
-        <v>122</v>
-      </c>
-      <c r="J4" t="s">
-        <v>116</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1437,10 +1437,10 @@
         <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -1455,13 +1455,13 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
+        <v>112</v>
+      </c>
+      <c r="I5" t="s">
+        <v>120</v>
+      </c>
+      <c r="J5" t="s">
         <v>114</v>
-      </c>
-      <c r="I5" t="s">
-        <v>122</v>
-      </c>
-      <c r="J5" t="s">
-        <v>116</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -1475,10 +1475,10 @@
         <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -1493,13 +1493,13 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I6" t="s">
+        <v>120</v>
+      </c>
+      <c r="J6" t="s">
         <v>114</v>
-      </c>
-      <c r="I6" t="s">
-        <v>122</v>
-      </c>
-      <c r="J6" t="s">
-        <v>116</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -1513,10 +1513,10 @@
         <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -1531,13 +1531,13 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I7" t="s">
+        <v>120</v>
+      </c>
+      <c r="J7" t="s">
         <v>114</v>
-      </c>
-      <c r="I7" t="s">
-        <v>122</v>
-      </c>
-      <c r="J7" t="s">
-        <v>116</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -1551,10 +1551,10 @@
         <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1569,13 +1569,13 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
@@ -1586,10 +1586,10 @@
         <v>87</v>
       </c>
       <c r="B9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D9">
         <v>3</v>
@@ -1604,13 +1604,13 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
@@ -1624,10 +1624,10 @@
         <v>89</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -1642,13 +1642,13 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
@@ -1662,10 +1662,10 @@
         <v>91</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -1680,13 +1680,13 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1718,13 +1718,13 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N12" t="b">
         <v>1</v>
@@ -1732,13 +1732,13 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -1753,13 +1753,13 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I13" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N13" t="b">
         <v>1</v>
@@ -1770,13 +1770,13 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1791,13 +1791,13 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
@@ -1808,10 +1808,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1826,13 +1826,13 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
+        <v>112</v>
+      </c>
+      <c r="I15" t="s">
+        <v>113</v>
+      </c>
+      <c r="J15" t="s">
         <v>114</v>
-      </c>
-      <c r="I15" t="s">
-        <v>115</v>
-      </c>
-      <c r="J15" t="s">
-        <v>116</v>
       </c>
       <c r="N15" t="b">
         <v>1</v>
@@ -1846,7 +1846,7 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1861,13 +1861,13 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J16" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
@@ -1881,7 +1881,7 @@
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1896,13 +1896,13 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I17" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
@@ -1916,7 +1916,7 @@
         <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1931,13 +1931,13 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
+        <v>133</v>
+      </c>
+      <c r="I18" t="s">
         <v>135</v>
       </c>
-      <c r="I18" t="s">
-        <v>137</v>
-      </c>
       <c r="J18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
@@ -1948,10 +1948,10 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1966,13 +1966,13 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I19" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J19" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N19" t="b">
         <v>1</v>
@@ -1980,13 +1980,13 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C20" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2001,13 +2001,13 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
@@ -2015,13 +2015,13 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B21" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C21" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H21" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N21" t="b">
         <v>1</v>
@@ -2050,13 +2050,13 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C22" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -2071,13 +2071,13 @@
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I22" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N22" t="b">
         <v>1</v>
@@ -2095,24 +2095,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
@@ -2121,10 +2121,10 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2517,7 +2517,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -2528,13 +2528,13 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -2542,13 +2542,13 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -2556,13 +2556,13 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2584,13 +2584,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>75</v>
@@ -2621,31 +2621,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2664,34 +2664,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>